<commit_message>
Enhance heuristic algorithms and data handling
- Increased maximum time limit from 30 to 100 in MainCall.jl to allow for longer processing.
- Improved route collection in HeuristicFunc.jl by ensuring empty routes are accounted for, enhancing the diversity of active routes.
- Adjusted the selection process for active routes to maintain a soft quota per base, optimizing the distribution of routes.
- Modified the random split ratio in Construction_Heuristic2 to favor larger subsets, improving the generation of candidate routes.
- Updated binary data files: LTM_demand.xlsx and Parameters.xlsx to reflect new demand and parameter configurations.
</commit_message>
<xml_diff>
--- a/inputData/LTM_demand.xlsx
+++ b/inputData/LTM_demand.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Kapta\Documents\DTU\Speciale\GitHubFiles\inputData\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3326953A-7A21-4AFF-A34D-8F5984C0D1F0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2B2E1A76-1D7B-4062-88EF-7093FC39BE5A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="PassengerGroups" sheetId="1" r:id="rId1"/>
@@ -444,7 +444,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F28"/>
+  <dimension ref="A1:F14"/>
   <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.35">
@@ -725,286 +725,6 @@
       </c>
       <c r="F14">
         <v>1</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A15">
-        <v>14</v>
-      </c>
-      <c r="B15">
-        <v>4</v>
-      </c>
-      <c r="C15">
-        <v>1</v>
-      </c>
-      <c r="D15">
-        <v>411</v>
-      </c>
-      <c r="E15">
-        <v>4</v>
-      </c>
-      <c r="F15">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A16">
-        <v>15</v>
-      </c>
-      <c r="B16">
-        <v>5</v>
-      </c>
-      <c r="C16">
-        <v>3</v>
-      </c>
-      <c r="D16">
-        <v>422</v>
-      </c>
-      <c r="E16">
-        <v>3</v>
-      </c>
-      <c r="F16">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A17">
-        <v>16</v>
-      </c>
-      <c r="B17">
-        <v>1</v>
-      </c>
-      <c r="C17">
-        <v>4</v>
-      </c>
-      <c r="D17">
-        <v>454</v>
-      </c>
-      <c r="E17">
-        <v>2</v>
-      </c>
-      <c r="F17">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A18">
-        <v>17</v>
-      </c>
-      <c r="B18">
-        <v>1</v>
-      </c>
-      <c r="C18">
-        <v>4</v>
-      </c>
-      <c r="D18">
-        <v>454</v>
-      </c>
-      <c r="E18">
-        <v>4</v>
-      </c>
-      <c r="F18">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A19">
-        <v>18</v>
-      </c>
-      <c r="B19">
-        <v>2</v>
-      </c>
-      <c r="C19">
-        <v>1</v>
-      </c>
-      <c r="D19">
-        <v>529</v>
-      </c>
-      <c r="E19">
-        <v>1</v>
-      </c>
-      <c r="F19">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A20">
-        <v>19</v>
-      </c>
-      <c r="B20">
-        <v>4</v>
-      </c>
-      <c r="C20">
-        <v>1</v>
-      </c>
-      <c r="D20">
-        <v>560</v>
-      </c>
-      <c r="E20">
-        <v>3</v>
-      </c>
-      <c r="F20">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A21">
-        <v>20</v>
-      </c>
-      <c r="B21">
-        <v>1</v>
-      </c>
-      <c r="C21">
-        <v>2</v>
-      </c>
-      <c r="D21">
-        <v>562</v>
-      </c>
-      <c r="E21">
-        <v>2</v>
-      </c>
-      <c r="F21">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A22">
-        <v>21</v>
-      </c>
-      <c r="B22">
-        <v>5</v>
-      </c>
-      <c r="C22">
-        <v>3</v>
-      </c>
-      <c r="D22">
-        <v>578</v>
-      </c>
-      <c r="E22">
-        <v>3</v>
-      </c>
-      <c r="F22">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A23">
-        <v>22</v>
-      </c>
-      <c r="B23">
-        <v>2</v>
-      </c>
-      <c r="C23">
-        <v>3</v>
-      </c>
-      <c r="D23">
-        <v>582</v>
-      </c>
-      <c r="E23">
-        <v>4</v>
-      </c>
-      <c r="F23">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A24">
-        <v>23</v>
-      </c>
-      <c r="B24">
-        <v>1</v>
-      </c>
-      <c r="C24">
-        <v>4</v>
-      </c>
-      <c r="D24">
-        <v>652</v>
-      </c>
-      <c r="E24">
-        <v>2</v>
-      </c>
-      <c r="F24">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A25">
-        <v>24</v>
-      </c>
-      <c r="B25">
-        <v>2</v>
-      </c>
-      <c r="C25">
-        <v>1</v>
-      </c>
-      <c r="D25">
-        <v>654</v>
-      </c>
-      <c r="E25">
-        <v>4</v>
-      </c>
-      <c r="F25">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A26">
-        <v>25</v>
-      </c>
-      <c r="B26">
-        <v>4</v>
-      </c>
-      <c r="C26">
-        <v>3</v>
-      </c>
-      <c r="D26">
-        <v>659</v>
-      </c>
-      <c r="E26">
-        <v>4</v>
-      </c>
-      <c r="F26">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A27">
-        <v>26</v>
-      </c>
-      <c r="B27">
-        <v>1</v>
-      </c>
-      <c r="C27">
-        <v>4</v>
-      </c>
-      <c r="D27">
-        <v>663</v>
-      </c>
-      <c r="E27">
-        <v>3</v>
-      </c>
-      <c r="F27">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.35">
-      <c r="A28">
-        <v>27</v>
-      </c>
-      <c r="B28">
-        <v>4</v>
-      </c>
-      <c r="C28">
-        <v>1</v>
-      </c>
-      <c r="D28">
-        <v>747</v>
-      </c>
-      <c r="E28">
-        <v>4</v>
-      </c>
-      <c r="F28">
-        <v>0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>